<commit_message>
feat: :memo: update absen
</commit_message>
<xml_diff>
--- a/TimesheetBankJakarta_Anggit_Ari_Utomo_2.xlsx
+++ b/TimesheetBankJakarta_Anggit_Ari_Utomo_2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\anggit\Documents\absen\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\anggit\absen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1310801A-EC35-460E-8356-3882AD47CC21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{227D4318-1055-4A54-B329-CC5383FBCD35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6043,11 +6043,15 @@
       <c r="D26" s="8">
         <v>0.70833333333333337</v>
       </c>
-      <c r="E26" s="105"/>
-      <c r="F26" s="8"/>
+      <c r="E26" s="105">
+        <v>0.33124999999999999</v>
+      </c>
+      <c r="F26" s="8">
+        <v>0.72430555555555554</v>
+      </c>
       <c r="G26" s="11">
         <f t="shared" ref="G26:G30" si="2">ROUND(MOD(F26-E26-TIME(1,0,0),1)*24,1)</f>
-        <v>23</v>
+        <v>8.4</v>
       </c>
       <c r="H26" s="14"/>
       <c r="I26" s="14" t="s">
@@ -6070,11 +6074,15 @@
       <c r="D27" s="8">
         <v>0.70833333333333337</v>
       </c>
-      <c r="E27" s="105"/>
-      <c r="F27" s="8"/>
+      <c r="E27" s="105">
+        <v>0.31111111111111112</v>
+      </c>
+      <c r="F27" s="8">
+        <v>0.73541666666666672</v>
+      </c>
       <c r="G27" s="11">
         <f t="shared" si="2"/>
-        <v>23</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="H27" s="14"/>
       <c r="I27" s="14" t="s">
@@ -6097,11 +6105,15 @@
       <c r="D28" s="8">
         <v>0.70833333333333337</v>
       </c>
-      <c r="E28" s="105"/>
-      <c r="F28" s="8"/>
+      <c r="E28" s="105">
+        <v>0.3263888888888889</v>
+      </c>
+      <c r="F28" s="8">
+        <v>0.74652777777777779</v>
+      </c>
       <c r="G28" s="11">
         <f t="shared" si="2"/>
-        <v>23</v>
+        <v>9.1</v>
       </c>
       <c r="H28" s="14"/>
       <c r="I28" s="14" t="s">
@@ -6124,11 +6136,15 @@
       <c r="D29" s="8">
         <v>0.70833333333333337</v>
       </c>
-      <c r="E29" s="105"/>
-      <c r="F29" s="8"/>
+      <c r="E29" s="105">
+        <v>0.34513888888888888</v>
+      </c>
+      <c r="F29" s="8">
+        <v>0.7270833333333333</v>
+      </c>
       <c r="G29" s="11">
         <f t="shared" si="2"/>
-        <v>23</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="H29" s="14"/>
       <c r="I29" s="14" t="s">
@@ -6151,11 +6167,13 @@
       <c r="D30" s="8">
         <v>0.70833333333333337</v>
       </c>
-      <c r="E30" s="105"/>
+      <c r="E30" s="105">
+        <v>0.3</v>
+      </c>
       <c r="F30" s="8"/>
       <c r="G30" s="11">
         <f t="shared" si="2"/>
-        <v>23</v>
+        <v>15.8</v>
       </c>
       <c r="H30" s="14"/>
       <c r="I30" s="14" t="s">
@@ -6385,7 +6403,7 @@
       <c r="F43" s="138"/>
       <c r="G43" s="18">
         <f>SUM(G9:G39)</f>
-        <v>301.39999999999998</v>
+        <v>237.1</v>
       </c>
       <c r="H43" s="19"/>
       <c r="I43" s="19"/>
@@ -6421,7 +6439,7 @@
       <c r="E45" s="25"/>
       <c r="F45" s="25"/>
       <c r="G45" s="26">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H45" s="129" t="s">
         <v>17</v>
@@ -6536,7 +6554,7 @@
       <c r="F51" s="25"/>
       <c r="G51" s="29">
         <f>G50/G45</f>
-        <v>1</v>
+        <v>1.0476190476190477</v>
       </c>
       <c r="H51" s="30" t="s">
         <v>26</v>
@@ -6583,7 +6601,7 @@
       <c r="F53" s="25"/>
       <c r="G53" s="27">
         <f>8*G45</f>
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="H53" s="35" t="s">
         <v>31</v>
@@ -6608,7 +6626,7 @@
       <c r="F54" s="2"/>
       <c r="G54" s="26">
         <f>G43</f>
-        <v>301.39999999999998</v>
+        <v>237.1</v>
       </c>
       <c r="H54" s="35" t="s">
         <v>33</v>
@@ -6633,7 +6651,7 @@
       <c r="F55" s="39"/>
       <c r="G55" s="40">
         <f>G54/G53</f>
-        <v>1.7124999999999999</v>
+        <v>1.4113095238095237</v>
       </c>
       <c r="H55" s="41" t="s">
         <v>35</v>
@@ -10325,24 +10343,16 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="58">
-    <mergeCell ref="J34:L34"/>
-    <mergeCell ref="J35:L35"/>
-    <mergeCell ref="J36:L36"/>
-    <mergeCell ref="J37:L37"/>
     <mergeCell ref="J13:L13"/>
     <mergeCell ref="J14:L14"/>
     <mergeCell ref="J15:L15"/>
     <mergeCell ref="J16:L16"/>
     <mergeCell ref="J26:L26"/>
-    <mergeCell ref="J27:L27"/>
-    <mergeCell ref="J28:L28"/>
-    <mergeCell ref="J29:L29"/>
-    <mergeCell ref="J30:L30"/>
+    <mergeCell ref="J22:L22"/>
+    <mergeCell ref="J23:L23"/>
     <mergeCell ref="J19:L19"/>
     <mergeCell ref="J20:L20"/>
     <mergeCell ref="J21:L21"/>
-    <mergeCell ref="J22:L22"/>
-    <mergeCell ref="J23:L23"/>
     <mergeCell ref="C63:D63"/>
     <mergeCell ref="E63:G63"/>
     <mergeCell ref="H63:J63"/>
@@ -10351,6 +10361,14 @@
     <mergeCell ref="H62:J62"/>
     <mergeCell ref="K62:L62"/>
     <mergeCell ref="C62:D62"/>
+    <mergeCell ref="J34:L34"/>
+    <mergeCell ref="J35:L35"/>
+    <mergeCell ref="J36:L36"/>
+    <mergeCell ref="J37:L37"/>
+    <mergeCell ref="J27:L27"/>
+    <mergeCell ref="J28:L28"/>
+    <mergeCell ref="J29:L29"/>
+    <mergeCell ref="J30:L30"/>
     <mergeCell ref="H7:H8"/>
     <mergeCell ref="I7:I8"/>
     <mergeCell ref="J7:L8"/>

</xml_diff>